<commit_message>
JAX Numpyro + diffrax implementation (#70)
</commit_message>
<xml_diff>
--- a/scripts/hyperoptimisation/results.xlsx
+++ b/scripts/hyperoptimisation/results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twa27/Documents/github/FluSight/Cornell_JHU-SCARCHhierarSIR/scripts/hyperoptimisation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5006C86B-0792-0D46-A25E-A17B0668E3AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3668F207-02D4-8C49-9AEF-8843F31ED720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="980" yWindow="880" windowWidth="28040" windowHeight="16240" xr2:uid="{2A525A24-CBD9-4142-97B4-C9C09D65775D}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>phi</t>
   </si>
@@ -62,6 +62,12 @@
   </si>
   <si>
     <t>reduction</t>
+  </si>
+  <si>
+    <t>Examples of artificially inflating noise with a GRW on the SIR model output:</t>
+  </si>
+  <si>
+    <t>sigma_grw</t>
   </si>
 </sst>
 </file>
@@ -3660,6 +3666,182 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>188812</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>241300</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Picture 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F91C9810-F2C3-F700-5156-E55E2F55D5F3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15047812" y="1447800"/>
+          <a:ext cx="4179988" cy="2997200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>203200</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>221369</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Picture 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E4A4018-0A7C-F4AA-9628-20F5BB1A1C87}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15062200" y="4457700"/>
+          <a:ext cx="4145669" cy="3111500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>26309</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>575796</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>50801</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="Picture 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB01EB3B-1518-AA3F-05E6-B754A70660AF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22072600" y="4496709"/>
+          <a:ext cx="4093696" cy="3072492"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>565736</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>203199</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>516222</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Picture 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EB098BB-6698-A037-85D0-6AD118B4FF8F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22028736" y="1422399"/>
+          <a:ext cx="4077986" cy="3060701"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3980,10 +4162,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2C7F92F-6776-B24A-A9FC-F25929B0C563}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:Z30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3997,7 +4179,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0.25</v>
       </c>
@@ -4011,7 +4193,7 @@
         <v>0.20382500000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>0.375</v>
       </c>
@@ -4025,7 +4207,7 @@
         <v>0.20455499999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>0.5</v>
       </c>
@@ -4039,7 +4221,7 @@
         <v>0.20483499999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>0.625</v>
       </c>
@@ -4063,7 +4245,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>0.75</v>
       </c>
@@ -4076,8 +4258,19 @@
       <c r="D6">
         <v>0.21549199999999999</v>
       </c>
+      <c r="S6" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="24" spans="4:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Y13" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z13">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="24" spans="4:26" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
         <v>4</v>
       </c>
@@ -4088,6 +4281,14 @@
         <v>6</v>
       </c>
     </row>
+    <row r="30" spans="4:26" x14ac:dyDescent="0.2">
+      <c r="Y30" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z30">
+        <v>0.01</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>